<commit_message>
Add new Excel session data for 2nd Ferdous session 879
</commit_message>
<xml_diff>
--- a/Sessions/2nd October session 3.xlsx
+++ b/Sessions/2nd October session 3.xlsx
@@ -548,8 +548,16 @@
           <t>null 2</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>01:15:18 AM</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
@@ -630,8 +638,16 @@
           <t>null 4</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>01:15:19 AM</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
@@ -753,8 +769,16 @@
           <t>null 7</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>01:15:24 AM</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
@@ -798,8 +822,16 @@
           <t>null 8</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>01:15:27 AM</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
@@ -843,8 +875,16 @@
           <t>null 9</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>01:15:30 AM</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
@@ -888,8 +928,16 @@
           <t>null 10</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>01:15:36 AM</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>

</xml_diff>